<commit_message>
Populate CI Register with defined configuration items
</commit_message>
<xml_diff>
--- a/docs/CI_Register.xlsx
+++ b/docs/CI_Register.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="140" windowWidth="15300" windowHeight="7090"/>
+    <workbookView xWindow="130" yWindow="490" windowWidth="18880" windowHeight="8740"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="CI_Register" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="80">
+  <si>
+    <t>CI ID</t>
+  </si>
   <si>
     <t>CI Name</t>
   </si>
@@ -31,22 +32,236 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Date Created</t>
+  </si>
+  <si>
+    <t>Last Modified</t>
+  </si>
+  <si>
+    <t>DOC-001</t>
+  </si>
+  <si>
+    <t>SCMP_v1.0.docx</t>
+  </si>
+  <si>
+    <t>v1.0</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Initial SCM plan</t>
+  </si>
+  <si>
+    <t>2025-12-21</t>
+  </si>
+  <si>
+    <t>DOC-002</t>
+  </si>
+  <si>
+    <t>CI_Register.xlsx</t>
+  </si>
+  <si>
+    <t>Tracks all configuration items</t>
+  </si>
+  <si>
+    <t>DOC-003</t>
+  </si>
+  <si>
+    <t>Requirements.docx</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>Functional &amp; non-functional requirements</t>
+  </si>
+  <si>
+    <t>DOC-004</t>
+  </si>
+  <si>
+    <t>User_Manual.docx</t>
+  </si>
+  <si>
+    <t>Instructions for students</t>
+  </si>
+  <si>
+    <t>DOC-005</t>
+  </si>
+  <si>
+    <t>Developer_Guide.docx</t>
+  </si>
+  <si>
+    <t>Guidelines for developers</t>
+  </si>
+  <si>
+    <t>DOC-006</t>
+  </si>
+  <si>
+    <t>Change_Request_Form.docx</t>
+  </si>
+  <si>
+    <t>CR submission template</t>
+  </si>
+  <si>
+    <t>DOC-007</t>
+  </si>
+  <si>
+    <t>Change_Log.xlsx</t>
+  </si>
+  <si>
+    <t>Tracks change requests</t>
+  </si>
+  <si>
+    <t>DOC-008</t>
+  </si>
+  <si>
+    <t>Configuration_Audit_Report.docx</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>PCA &amp; FCA report</t>
+  </si>
+  <si>
+    <t>DOC-009</t>
+  </si>
+  <si>
+    <t>Team_Work_Distribution.docx</t>
+  </si>
+  <si>
+    <t>Team contribution record</t>
+  </si>
+  <si>
+    <t>SRC-001</t>
+  </si>
+  <si>
+    <t>src/student_record.py</t>
+  </si>
+  <si>
+    <t>Source Code</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Core student record logic</t>
+  </si>
+  <si>
+    <t>SRC-002</t>
+  </si>
+  <si>
+    <t>src/database.json</t>
+  </si>
+  <si>
+    <t>Student data storage</t>
+  </si>
+  <si>
+    <t>SRC-003</t>
+  </si>
+  <si>
+    <t>src/login_page.html</t>
+  </si>
+  <si>
+    <t>Login page</t>
+  </si>
+  <si>
+    <t>SRC-004</t>
+  </si>
+  <si>
+    <t>src/dashboard.html</t>
+  </si>
+  <si>
+    <t>Student dashboard</t>
+  </si>
+  <si>
+    <t>TEST-001</t>
+  </si>
+  <si>
+    <t>tests/test_student_record.xlsx</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Student record test cases</t>
+  </si>
+  <si>
+    <t>TEST-002</t>
+  </si>
+  <si>
+    <t>tests/test_results.xlsx</t>
+  </si>
+  <si>
+    <t>Test results</t>
+  </si>
+  <si>
+    <t>TEST-003</t>
+  </si>
+  <si>
+    <t>tests/login_test.xlsx</t>
+  </si>
+  <si>
+    <t>Login tests</t>
+  </si>
+  <si>
+    <t>REL-001</t>
+  </si>
+  <si>
+    <t>releases/v1.0.zip</t>
+  </si>
+  <si>
+    <t>Release</t>
+  </si>
+  <si>
+    <t>Initial release</t>
+  </si>
+  <si>
+    <t>REL-002</t>
+  </si>
+  <si>
+    <t>releases/v1.1.zip</t>
+  </si>
+  <si>
+    <t>Post-change release</t>
+  </si>
+  <si>
+    <t>Dagmawit Gebreweld</t>
+  </si>
+  <si>
+    <t>Danayt Esayas</t>
+  </si>
+  <si>
+    <t>Dagmawit Negash</t>
+  </si>
+  <si>
+    <t>Birhan Aklil</t>
+  </si>
+  <si>
+    <t>Dagm Taye</t>
+  </si>
+  <si>
+    <t>Burka Labsi</t>
+  </si>
+  <si>
+    <t>Delina Mulubirhan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -74,17 +289,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -168,7 +380,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -203,7 +414,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -380,11 +590,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="30.08984375" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" customWidth="1"/>
+    <col min="4" max="4" width="23.7265625" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="13.36328125" customWidth="1"/>
+    <col min="7" max="7" width="37.1796875" customWidth="1"/>
+    <col min="8" max="8" width="14.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -399,26 +618,527 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" t="s">
+        <v>49</v>
+      </c>
+      <c r="H12" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" t="s">
+        <v>62</v>
+      </c>
+      <c r="H16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H17" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" t="s">
+        <v>69</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" t="s">
+        <v>37</v>
+      </c>
+      <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>